<commit_message>
adjust web app, add more models and upload label automatically
</commit_message>
<xml_diff>
--- a/V-Unet/summary.xlsx
+++ b/V-Unet/summary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rosehulman-my.sharepoint.com/personal/yec1_rose-hulman_edu/Documents/Rose-Hulman/course/CSSE/CSSE416/project/CSSE416-breast-image-segmentation/V-Unet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="159" documentId="11_F25DC773A252ABDACC10485231197CC85BDE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6831C0EF-243E-4CED-BBDE-A42170BD1F9A}"/>
+  <xr:revisionPtr revIDLastSave="167" documentId="11_F25DC773A252ABDACC10485231197CC85BDE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AA975569-CF44-490C-A852-34B7AF6736C1}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="780" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -151,7 +151,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -162,6 +162,13 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -202,18 +209,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -231,6 +241,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -525,11 +539,11 @@
       <c r="I2" s="1"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
@@ -547,19 +561,19 @@
       <c r="I4" s="1"/>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="2" t="s">
         <v>6</v>
       </c>
       <c r="G5" s="1"/>
@@ -567,19 +581,19 @@
       <c r="I5" s="1"/>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="2">
         <v>0.34699999999999998</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="2">
         <v>0.23899999999999999</v>
       </c>
-      <c r="E6" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="F6" s="3" t="s">
+      <c r="E6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G6" s="1"/>
@@ -587,19 +601,19 @@
       <c r="I6" s="1"/>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="5">
         <v>0.41499999999999998</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="5">
         <v>0.29799999999999999</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="5" t="s">
         <v>10</v>
       </c>
       <c r="G7" s="1"/>
@@ -607,19 +621,19 @@
       <c r="I7" s="1"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="2">
         <v>0.36099999999999999</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="2">
         <v>0.27100000000000002</v>
       </c>
-      <c r="E8" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="F8" s="3" t="s">
+      <c r="E8" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>12</v>
       </c>
       <c r="G8" s="1"/>
@@ -627,19 +641,19 @@
       <c r="I8" s="1"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="3">
+      <c r="C9" s="5">
         <v>0.46300000000000002</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="5">
         <v>0.34200000000000003</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="F9" s="5" t="s">
         <v>14</v>
       </c>
       <c r="G9" s="1"/>
@@ -647,19 +661,19 @@
       <c r="I9" s="1"/>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="2">
         <v>0.433</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="2">
         <v>0.313</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="F10" s="2" t="s">
         <v>16</v>
       </c>
       <c r="G10" s="1"/>
@@ -667,19 +681,19 @@
       <c r="I10" s="1"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C11" s="2">
         <v>0.35199999999999998</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D11" s="2">
         <v>0.25900000000000001</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="F11" s="2" t="s">
         <v>18</v>
       </c>
       <c r="G11" s="1"/>
@@ -729,19 +743,19 @@
       <c r="I15" s="1"/>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E16" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="F16" s="2" t="s">
         <v>6</v>
       </c>
       <c r="G16" s="1"/>
@@ -749,19 +763,19 @@
       <c r="I16" s="1"/>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C17" s="3">
+      <c r="C17" s="5">
         <v>0.40400000000000003</v>
       </c>
-      <c r="D17" s="3">
+      <c r="D17" s="5">
         <v>0.28699999999999998</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="E17" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="F17" s="5" t="s">
         <v>21</v>
       </c>
       <c r="G17" s="1"/>
@@ -769,96 +783,96 @@
       <c r="I17" s="1"/>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C18" s="3">
+      <c r="C18" s="2">
         <v>0.40699999999999997</v>
       </c>
-      <c r="D18" s="3">
+      <c r="D18" s="2">
         <v>0.30599999999999999</v>
       </c>
-      <c r="E18" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="F18" s="3" t="s">
+      <c r="E18" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F18" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C19" s="3">
+      <c r="C19" s="5">
         <v>0.40799999999999997</v>
       </c>
-      <c r="D19" s="3">
+      <c r="D19" s="5">
         <v>0.30399999999999999</v>
       </c>
-      <c r="E19" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="F19" s="3" t="s">
+      <c r="E19" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F19" s="5" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C20" s="3">
+      <c r="C20" s="2">
         <v>0.44500000000000001</v>
       </c>
-      <c r="D20" s="3">
+      <c r="D20" s="2">
         <v>0.34499999999999997</v>
       </c>
-      <c r="E20" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="F20" s="3" t="s">
+      <c r="E20" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F20" s="2" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C21" s="3">
+      <c r="C21" s="2">
         <v>0.42199999999999999</v>
       </c>
-      <c r="D21" s="3">
+      <c r="D21" s="2">
         <v>0.317</v>
       </c>
-      <c r="E21" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="F21" s="3" t="s">
+      <c r="E21" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F21" s="2" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C22" s="3">
+      <c r="C22" s="2">
         <v>0.34100000000000003</v>
       </c>
-      <c r="D22" s="3">
+      <c r="D22" s="2">
         <v>0.246</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="E22" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F22" s="3" t="s">
+      <c r="F22" s="2" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
     </row>
@@ -870,121 +884,121 @@
       <c r="F27" s="1"/>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B28" s="3" t="s">
+      <c r="B28" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="C28" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D28" s="3" t="s">
+      <c r="D28" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E28" s="3" t="s">
+      <c r="E28" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F28" s="3" t="s">
+      <c r="F28" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B29" s="3" t="s">
+      <c r="B29" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C29" s="3">
+      <c r="C29" s="5">
         <v>0.38300000000000001</v>
       </c>
-      <c r="D29" s="3">
+      <c r="D29" s="5">
         <v>0.308</v>
       </c>
-      <c r="E29" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="F29" s="3" t="s">
+      <c r="E29" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F29" s="5" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C30" s="3">
+      <c r="C30" s="2">
         <v>0.439</v>
       </c>
-      <c r="D30" s="3">
+      <c r="D30" s="2">
         <v>0.35299999999999998</v>
       </c>
-      <c r="E30" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="F30" s="3" t="s">
+      <c r="E30" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F30" s="2" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B31" s="3" t="s">
+      <c r="B31" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C31" s="3">
+      <c r="C31" s="2">
         <v>0.36899999999999999</v>
       </c>
-      <c r="D31" s="3">
+      <c r="D31" s="2">
         <v>0.29399999999999998</v>
       </c>
-      <c r="E31" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="F31" s="3" t="s">
+      <c r="E31" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F31" s="2" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B32" s="3" t="s">
+      <c r="B32" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C32" s="3">
+      <c r="C32" s="2">
         <v>0.45600000000000002</v>
       </c>
-      <c r="D32" s="3">
+      <c r="D32" s="2">
         <v>0.38400000000000001</v>
       </c>
-      <c r="E32" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="F32" s="3" t="s">
+      <c r="E32" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F32" s="2" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B33" s="3" t="s">
+      <c r="B33" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C33" s="3">
+      <c r="C33" s="5">
         <v>0.38800000000000001</v>
       </c>
-      <c r="D33" s="3">
+      <c r="D33" s="5">
         <v>0.309</v>
       </c>
-      <c r="E33" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="F33" s="3" t="s">
+      <c r="E33" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F33" s="5" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="34" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B34" s="3" t="s">
+      <c r="B34" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C34" s="3">
+      <c r="C34" s="2">
         <v>0.39400000000000002</v>
       </c>
-      <c r="D34" s="3">
+      <c r="D34" s="2">
         <v>0.32</v>
       </c>
-      <c r="E34" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="F34" s="3" t="s">
+      <c r="E34" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F34" s="2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1005,121 +1019,121 @@
       <c r="F39" s="1"/>
     </row>
     <row r="40" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B40" s="3" t="s">
+      <c r="B40" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C40" s="3" t="s">
+      <c r="C40" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D40" s="3" t="s">
+      <c r="D40" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E40" s="3" t="s">
+      <c r="E40" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F40" s="3" t="s">
+      <c r="F40" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="41" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B41" s="3" t="s">
+      <c r="B41" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C41" s="3">
+      <c r="C41" s="2">
         <v>0.441</v>
       </c>
-      <c r="D41" s="3">
+      <c r="D41" s="2">
         <v>0.36899999999999999</v>
       </c>
-      <c r="E41" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="F41" s="3" t="s">
+      <c r="E41" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F41" s="2" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="42" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B42" s="3" t="s">
+      <c r="B42" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C42" s="3">
+      <c r="C42" s="2">
         <v>0.38</v>
       </c>
-      <c r="D42" s="3">
+      <c r="D42" s="2">
         <v>0.30499999999999999</v>
       </c>
-      <c r="E42" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="F42" s="3" t="s">
+      <c r="E42" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F42" s="2" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="43" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B43" s="3" t="s">
+      <c r="B43" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C43" s="3">
+      <c r="C43" s="5">
         <v>0.38</v>
       </c>
-      <c r="D43" s="3">
+      <c r="D43" s="5">
         <v>0.30499999999999999</v>
       </c>
-      <c r="E43" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="F43" s="3" t="s">
+      <c r="E43" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F43" s="5" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="44" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B44" s="3" t="s">
+      <c r="B44" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C44" s="3">
+      <c r="C44" s="5">
         <v>0.44600000000000001</v>
       </c>
-      <c r="D44" s="3">
+      <c r="D44" s="5">
         <v>0.374</v>
       </c>
-      <c r="E44" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="F44" s="3" t="s">
+      <c r="E44" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F44" s="5" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="45" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B45" s="3" t="s">
+      <c r="B45" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C45" s="3">
+      <c r="C45" s="2">
         <v>0.42699999999999999</v>
       </c>
-      <c r="D45" s="3">
+      <c r="D45" s="2">
         <v>0.35</v>
       </c>
-      <c r="E45" s="3" t="s">
+      <c r="E45" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F45" s="3" t="s">
+      <c r="F45" s="2" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="46" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B46" s="3" t="s">
+      <c r="B46" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C46" s="3">
+      <c r="C46" s="2">
         <v>0.35199999999999998</v>
       </c>
-      <c r="D46" s="3">
+      <c r="D46" s="2">
         <v>0.28100000000000003</v>
       </c>
-      <c r="E46" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="F46" s="3" t="s">
+      <c r="E46" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F46" s="2" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>